<commit_message>
now its working, new comp june 2026
</commit_message>
<xml_diff>
--- a/src/AlgoComposition.xlsx
+++ b/src/AlgoComposition.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
@@ -14,8 +14,8 @@
     <sheet name="2015" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">'2015'!$A$1:$E$43</definedName>
-    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'2020'!$A$1:$E$43</definedName>
+    <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">'2015'!$A$1:$E$48</definedName>
+    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'2020'!$A$1:$E$48</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="96">
   <si>
     <t xml:space="preserve">Symbol</t>
   </si>
@@ -104,6 +104,30 @@
     <t xml:space="preserve">Apple Inc.</t>
   </si>
   <si>
+    <t xml:space="preserve">AMAT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Applied Materials</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SNDK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sandisk Corporation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">APH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apollo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INTU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Intuit</t>
+  </si>
+  <si>
     <t xml:space="preserve">GRMN</t>
   </si>
   <si>
@@ -116,27 +140,21 @@
     <t xml:space="preserve">Shopify Inc.</t>
   </si>
   <si>
+    <t xml:space="preserve">AMZN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Inc.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Micron</t>
+  </si>
+  <si>
     <t xml:space="preserve">GOOG</t>
   </si>
   <si>
     <t xml:space="preserve">Google Inc.</t>
   </si>
   <si>
-    <t xml:space="preserve">AMZN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Amazon Inc.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Micron</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SNDK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sandisk Corporation</t>
-  </si>
-  <si>
     <t xml:space="preserve">HOOD</t>
   </si>
   <si>
@@ -155,9 +173,6 @@
     <t xml:space="preserve">Autozone</t>
   </si>
   <si>
-    <t xml:space="preserve">APH</t>
-  </si>
-  <si>
     <t xml:space="preserve">MA</t>
   </si>
   <si>
@@ -179,12 +194,6 @@
     <t xml:space="preserve">Pepsi</t>
   </si>
   <si>
-    <t xml:space="preserve">INTU</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Intuit</t>
-  </si>
-  <si>
     <t xml:space="preserve">AJG</t>
   </si>
   <si>
@@ -222,6 +231,12 @@
   </si>
   <si>
     <t xml:space="preserve">Visa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DELL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dell</t>
   </si>
   <si>
     <t xml:space="preserve">Apple</t>
@@ -310,7 +325,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -348,6 +363,13 @@
     </font>
     <font>
       <sz val="12"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFCACACA"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
@@ -420,7 +442,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -446,6 +468,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -481,6 +507,66 @@
       </fill>
     </dxf>
   </dxfs>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008000"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FFCACACA"/>
+      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FF9999FF"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FF660066"/>
+      <rgbColor rgb="FFFF8080"/>
+      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FF00CCFF"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FF99CCFF"/>
+      <rgbColor rgb="FFFF99CC"/>
+      <rgbColor rgb="FFCC99FF"/>
+      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FF3366FF"/>
+      <rgbColor rgb="FF33CCCC"/>
+      <rgbColor rgb="FF99CC00"/>
+      <rgbColor rgb="FFFFCC00"/>
+      <rgbColor rgb="FFFF9900"/>
+      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF339966"/>
+      <rgbColor rgb="FF003300"/>
+      <rgbColor rgb="FF333300"/>
+      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FF333399"/>
+      <rgbColor rgb="FF333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -500,37 +586,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -930,7 +1016,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J62"/>
+  <dimension ref="A1:J67"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14.02"/>
@@ -960,7 +1046,7 @@
         <v>25</v>
       </c>
       <c r="B2" s="5" t="n">
-        <v>46091</v>
+        <v>46175</v>
       </c>
       <c r="C2" s="5" t="n">
         <v>55146</v>
@@ -978,7 +1064,7 @@
         <v>27</v>
       </c>
       <c r="B3" s="5" t="n">
-        <v>46091</v>
+        <v>46139</v>
       </c>
       <c r="C3" s="5" t="n">
         <v>55146</v>
@@ -996,10 +1082,10 @@
         <v>29</v>
       </c>
       <c r="B4" s="5" t="n">
-        <v>46077</v>
+        <v>46139</v>
       </c>
       <c r="C4" s="5" t="n">
-        <v>46090</v>
+        <v>55146</v>
       </c>
       <c r="D4" s="6" t="n">
         <f aca="false">1/7</f>
@@ -1011,28 +1097,28 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="B5" s="5" t="n">
-        <v>46077</v>
+        <v>46139</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>55146</v>
+        <v>46174</v>
       </c>
       <c r="D5" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>32</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="B6" s="5" t="n">
-        <v>45903</v>
+        <v>46139</v>
       </c>
       <c r="C6" s="5" t="n">
         <v>55146</v>
@@ -1042,228 +1128,229 @@
         <v>0.142857142857143</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="I6" s="7"/>
+        <v>32</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>5</v>
+        <v>33</v>
       </c>
       <c r="B7" s="5" t="n">
-        <v>45965</v>
+        <v>46091</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>55146</v>
+        <v>46138</v>
       </c>
       <c r="D7" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="I7" s="7"/>
+        <v>34</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
       <c r="B8" s="5" t="n">
-        <v>45748</v>
+        <v>46091</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>55146</v>
+        <v>46138</v>
       </c>
       <c r="D8" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>10</v>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="H8" s="7"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="B9" s="5" t="n">
         <v>46077</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>55146</v>
+        <v>46138</v>
       </c>
       <c r="D9" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>24</v>
+        <v>38</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B10" s="5" t="n">
-        <v>45965</v>
+        <v>45903</v>
       </c>
       <c r="C10" s="5" t="n">
-        <v>46090</v>
+        <v>55146</v>
       </c>
       <c r="D10" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="J10" s="7"/>
+        <v>39</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="B11" s="5" t="n">
-        <v>45931</v>
+        <v>45965</v>
       </c>
       <c r="C11" s="5" t="n">
-        <v>46076</v>
+        <v>55146</v>
       </c>
       <c r="D11" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J11" s="7"/>
+        <v>6</v>
+      </c>
+      <c r="I11" s="8"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="B12" s="5" t="n">
-        <v>45931</v>
+        <v>45748</v>
       </c>
       <c r="C12" s="5" t="n">
-        <v>46076</v>
+        <v>55146</v>
       </c>
       <c r="D12" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="J12" s="7"/>
+        <v>10</v>
+      </c>
+      <c r="I12" s="8"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="B13" s="5" t="n">
-        <v>46061</v>
+        <v>46077</v>
       </c>
       <c r="C13" s="5" t="n">
-        <v>46076</v>
+        <v>46138</v>
       </c>
       <c r="D13" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B14" s="5" t="n">
-        <v>46048</v>
+        <v>46077</v>
       </c>
       <c r="C14" s="5" t="n">
-        <v>46060</v>
+        <v>46090</v>
       </c>
       <c r="D14" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="B15" s="5" t="n">
-        <v>45993</v>
+        <v>45965</v>
       </c>
       <c r="C15" s="5" t="n">
-        <v>46047</v>
+        <v>46090</v>
       </c>
       <c r="D15" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>22</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="J15" s="8"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
       <c r="B16" s="5" t="n">
-        <v>45903</v>
+        <v>45931</v>
       </c>
       <c r="C16" s="5" t="n">
-        <v>45992</v>
+        <v>46076</v>
       </c>
       <c r="D16" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>39</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="J16" s="8"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B17" s="5" t="n">
         <v>45931</v>
       </c>
       <c r="C17" s="5" t="n">
-        <v>45964</v>
+        <v>46076</v>
       </c>
       <c r="D17" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>19</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="J17" s="8"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="B18" s="5" t="n">
-        <v>45931</v>
+        <v>46061</v>
       </c>
       <c r="C18" s="5" t="n">
-        <v>45964</v>
+        <v>46076</v>
       </c>
       <c r="D18" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1271,82 +1358,82 @@
         <v>42</v>
       </c>
       <c r="B19" s="5" t="n">
-        <v>45778</v>
+        <v>46048</v>
       </c>
       <c r="C19" s="5" t="n">
-        <v>45930</v>
+        <v>46060</v>
       </c>
       <c r="D19" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B20" s="5" t="n">
-        <v>45839</v>
+        <v>45993</v>
       </c>
       <c r="C20" s="5" t="n">
-        <v>45930</v>
+        <v>46047</v>
       </c>
       <c r="D20" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B21" s="5" t="n">
-        <v>45839</v>
+        <v>45903</v>
       </c>
       <c r="C21" s="5" t="n">
-        <v>45930</v>
+        <v>45992</v>
       </c>
       <c r="D21" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>45</v>
+        <v>19</v>
       </c>
       <c r="B22" s="5" t="n">
-        <v>45839</v>
+        <v>45931</v>
       </c>
       <c r="C22" s="5" t="n">
-        <v>45930</v>
+        <v>45964</v>
       </c>
       <c r="D22" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>46</v>
+        <v>19</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B23" s="5" t="n">
-        <v>45870</v>
+        <v>45931</v>
       </c>
       <c r="C23" s="5" t="n">
-        <v>45902</v>
+        <v>45964</v>
       </c>
       <c r="D23" s="6" t="n">
         <f aca="false">1/7</f>
@@ -1358,383 +1445,453 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="B24" s="5" t="n">
-        <v>45870</v>
+        <v>45778</v>
       </c>
       <c r="C24" s="5" t="n">
-        <v>45902</v>
+        <v>45930</v>
       </c>
       <c r="D24" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>49</v>
+        <v>29</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="B25" s="5" t="n">
-        <v>45692</v>
+        <v>45839</v>
       </c>
       <c r="C25" s="5" t="n">
-        <v>45869</v>
+        <v>45930</v>
       </c>
       <c r="D25" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>51</v>
+        <v>34</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>5</v>
+        <v>48</v>
       </c>
       <c r="B26" s="5" t="n">
-        <v>45653</v>
+        <v>45839</v>
       </c>
       <c r="C26" s="5" t="n">
-        <v>45869</v>
+        <v>45930</v>
       </c>
       <c r="D26" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>6</v>
+        <v>49</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B27" s="5" t="n">
-        <v>45748</v>
+        <v>45839</v>
       </c>
       <c r="C27" s="5" t="n">
-        <v>45838</v>
+        <v>45930</v>
       </c>
       <c r="D27" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B28" s="5" t="n">
-        <v>45778</v>
+        <v>45870</v>
       </c>
       <c r="C28" s="5" t="n">
-        <v>45838</v>
+        <v>45902</v>
       </c>
       <c r="D28" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B29" s="5" t="n">
-        <v>45811</v>
+        <v>45870</v>
       </c>
       <c r="C29" s="5" t="n">
-        <v>45838</v>
+        <v>45902</v>
       </c>
       <c r="D29" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>57</v>
+        <v>31</v>
       </c>
       <c r="B30" s="5" t="n">
-        <v>45778</v>
+        <v>45692</v>
       </c>
       <c r="C30" s="5" t="n">
-        <v>45810</v>
+        <v>45869</v>
       </c>
       <c r="D30" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>57</v>
+        <v>32</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="B31" s="5" t="n">
-        <v>45748</v>
+        <v>45653</v>
       </c>
       <c r="C31" s="5" t="n">
-        <v>45777</v>
+        <v>45869</v>
       </c>
       <c r="D31" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B32" s="5" t="n">
-        <v>45692</v>
+        <v>45748</v>
       </c>
       <c r="C32" s="5" t="n">
-        <v>45777</v>
+        <v>45838</v>
       </c>
       <c r="D32" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="B33" s="5" t="n">
-        <v>45748</v>
+        <v>45778</v>
       </c>
       <c r="C33" s="5" t="n">
-        <v>45777</v>
+        <v>45838</v>
       </c>
       <c r="D33" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>23</v>
+        <v>58</v>
       </c>
       <c r="B34" s="5" t="n">
-        <v>45653</v>
+        <v>45811</v>
       </c>
       <c r="C34" s="5" t="n">
-        <v>45747</v>
+        <v>45838</v>
       </c>
       <c r="D34" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>24</v>
+        <v>59</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="B35" s="5" t="n">
-        <v>45653</v>
+        <v>45778</v>
       </c>
       <c r="C35" s="5" t="n">
-        <v>45747</v>
+        <v>45810</v>
       </c>
       <c r="D35" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="B36" s="5" t="n">
-        <v>45660</v>
+        <v>45748</v>
       </c>
       <c r="C36" s="5" t="n">
-        <v>45747</v>
+        <v>45777</v>
       </c>
       <c r="D36" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="B37" s="5" t="n">
-        <v>45660</v>
+        <v>45692</v>
       </c>
       <c r="C37" s="5" t="n">
-        <v>45747</v>
+        <v>45777</v>
       </c>
       <c r="D37" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
-        <v>29</v>
+        <v>63</v>
       </c>
       <c r="B38" s="5" t="n">
-        <v>45660</v>
+        <v>45748</v>
       </c>
       <c r="C38" s="5" t="n">
-        <v>45691</v>
+        <v>45777</v>
       </c>
       <c r="D38" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>30</v>
+        <v>64</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="B39" s="5" t="n">
-        <v>45660</v>
+        <v>45653</v>
       </c>
       <c r="C39" s="5" t="n">
-        <v>45691</v>
+        <v>45747</v>
       </c>
       <c r="D39" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
-        <v>17</v>
+        <v>37</v>
       </c>
       <c r="B40" s="5" t="n">
         <v>45653</v>
       </c>
       <c r="C40" s="5" t="n">
-        <v>45659</v>
+        <v>45747</v>
       </c>
       <c r="D40" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>18</v>
+        <v>65</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="s">
-        <v>15</v>
+        <v>33</v>
       </c>
       <c r="B41" s="5" t="n">
-        <v>45653</v>
+        <v>45660</v>
       </c>
       <c r="C41" s="5" t="n">
-        <v>45659</v>
+        <v>45747</v>
       </c>
       <c r="D41" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>16</v>
+        <v>34</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="s">
-        <v>19</v>
+        <v>50</v>
       </c>
       <c r="B42" s="5" t="n">
-        <v>45653</v>
+        <v>45660</v>
       </c>
       <c r="C42" s="5" t="n">
-        <v>45659</v>
+        <v>45747</v>
       </c>
       <c r="D42" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>19</v>
+        <v>51</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="4" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="B43" s="5" t="n">
+        <v>45660</v>
+      </c>
+      <c r="C43" s="5" t="n">
+        <v>45691</v>
+      </c>
+      <c r="D43" s="6" t="n">
+        <f aca="false">1/7</f>
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E43" s="6" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>45660</v>
+      </c>
+      <c r="C44" s="5" t="n">
+        <v>45691</v>
+      </c>
+      <c r="D44" s="6" t="n">
+        <f aca="false">1/7</f>
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E44" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B45" s="5" t="n">
         <v>45653</v>
       </c>
-      <c r="C43" s="5" t="n">
+      <c r="C45" s="5" t="n">
         <v>45659</v>
       </c>
-      <c r="D43" s="6" t="n">
-        <f aca="false">1/7</f>
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E43" s="6" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="5"/>
-      <c r="B44" s="5"/>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="5"/>
-      <c r="B45" s="5"/>
+      <c r="D45" s="6" t="n">
+        <f aca="false">1/7</f>
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E45" s="6" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="5"/>
-      <c r="B46" s="5"/>
+      <c r="A46" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>45653</v>
+      </c>
+      <c r="C46" s="5" t="n">
+        <v>45659</v>
+      </c>
+      <c r="D46" s="6" t="n">
+        <f aca="false">1/7</f>
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E46" s="6" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="5"/>
-      <c r="B47" s="5"/>
+      <c r="A47" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>45653</v>
+      </c>
+      <c r="C47" s="5" t="n">
+        <v>45659</v>
+      </c>
+      <c r="D47" s="6" t="n">
+        <f aca="false">1/7</f>
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E47" s="6" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="5"/>
-      <c r="B48" s="5"/>
+      <c r="A48" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>45653</v>
+      </c>
+      <c r="C48" s="5" t="n">
+        <v>45659</v>
+      </c>
+      <c r="D48" s="6" t="n">
+        <f aca="false">1/7</f>
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E48" s="6" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="5"/>
@@ -1792,8 +1949,28 @@
       <c r="A62" s="5"/>
       <c r="B62" s="5"/>
     </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="5"/>
+      <c r="B63" s="5"/>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="5"/>
+      <c r="B64" s="5"/>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="5"/>
+      <c r="B65" s="5"/>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="5"/>
+      <c r="B66" s="5"/>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="5"/>
+      <c r="B67" s="5"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E43"/>
+  <autoFilter ref="A1:E48"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -1810,7 +1987,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I60"/>
+  <dimension ref="A1:I65"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15.02"/>
@@ -1832,7 +2009,7 @@
       <c r="D1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" s="9" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1841,7 +2018,7 @@
         <v>27</v>
       </c>
       <c r="B2" s="5" t="n">
-        <v>46091</v>
+        <v>46140</v>
       </c>
       <c r="C2" s="5" t="n">
         <v>55146</v>
@@ -1853,39 +2030,37 @@
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
-      <c r="F2" s="6"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="B3" s="5" t="n">
-        <v>46091</v>
+        <v>46140</v>
       </c>
       <c r="C3" s="5" t="n">
         <v>55146</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E3" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
-      <c r="F3" s="6"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B4" s="5" t="n">
-        <v>45965</v>
+        <v>46140</v>
       </c>
       <c r="C4" s="5" t="n">
         <v>55146</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>65</v>
+        <v>26</v>
       </c>
       <c r="E4" s="6" t="n">
         <f aca="false">1/7</f>
@@ -1894,16 +2069,16 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>5</v>
+        <v>68</v>
       </c>
       <c r="B5" s="5" t="n">
-        <v>45931</v>
+        <v>46140</v>
       </c>
       <c r="C5" s="5" t="n">
         <v>55146</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="E5" s="6" t="n">
         <f aca="false">1/7</f>
@@ -1912,16 +2087,16 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B6" s="5" t="n">
-        <v>45748</v>
+        <v>46140</v>
       </c>
       <c r="C6" s="5" t="n">
         <v>55146</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>67</v>
+        <v>12</v>
       </c>
       <c r="E6" s="6" t="n">
         <f aca="false">1/7</f>
@@ -1930,53 +2105,55 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>48</v>
+        <v>35</v>
       </c>
       <c r="B7" s="5" t="n">
-        <v>46061</v>
+        <v>46091</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>55146</v>
+        <v>46140</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>68</v>
+        <v>36</v>
       </c>
       <c r="E7" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
+      <c r="F7" s="6"/>
+      <c r="G7" s="7"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
-        <v>31</v>
+      <c r="A8" s="4" t="s">
+        <v>33</v>
       </c>
       <c r="B8" s="5" t="n">
-        <v>46073</v>
+        <v>46091</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>55146</v>
+        <v>46140</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>69</v>
+        <v>34</v>
       </c>
       <c r="E8" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
-      <c r="H8" s="7"/>
+      <c r="F8" s="6"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="B9" s="5" t="n">
-        <v>45993</v>
+        <v>45965</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>46091</v>
+        <v>46140</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>12</v>
+        <v>70</v>
       </c>
       <c r="E9" s="6" t="n">
         <f aca="false">1/7</f>
@@ -1984,56 +2161,53 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="s">
-        <v>29</v>
+      <c r="A10" s="4" t="s">
+        <v>5</v>
       </c>
       <c r="B10" s="5" t="n">
-        <v>46073</v>
+        <v>45931</v>
       </c>
       <c r="C10" s="5" t="n">
-        <v>46091</v>
+        <v>55146</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>30</v>
+        <v>71</v>
       </c>
       <c r="E10" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
-      <c r="H10" s="7"/>
-      <c r="I10" s="7"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="B11" s="5" t="n">
-        <v>45931</v>
+        <v>45748</v>
       </c>
       <c r="C11" s="5" t="n">
-        <v>46072</v>
+        <v>55146</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>18</v>
+        <v>72</v>
       </c>
       <c r="E11" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
-      <c r="I11" s="7"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>34</v>
+        <v>53</v>
       </c>
       <c r="B12" s="5" t="n">
         <v>46061</v>
       </c>
       <c r="C12" s="5" t="n">
-        <v>46072</v>
+        <v>46140</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>35</v>
+        <v>73</v>
       </c>
       <c r="E12" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2041,35 +2215,36 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
-        <v>13</v>
+      <c r="A13" s="5" t="s">
+        <v>37</v>
       </c>
       <c r="B13" s="5" t="n">
-        <v>45993</v>
+        <v>46073</v>
       </c>
       <c r="C13" s="5" t="n">
-        <v>46060</v>
+        <v>46140</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>14</v>
+        <v>74</v>
       </c>
       <c r="E13" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
+      <c r="H13" s="8"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="B14" s="5" t="n">
-        <v>45931</v>
+        <v>45993</v>
       </c>
       <c r="C14" s="5" t="n">
-        <v>46060</v>
+        <v>46091</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="E14" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2077,53 +2252,56 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="5" t="s">
         <v>40</v>
       </c>
       <c r="B15" s="5" t="n">
-        <v>45903</v>
+        <v>46073</v>
       </c>
       <c r="C15" s="5" t="n">
-        <v>45992</v>
+        <v>46091</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="E15" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
+      <c r="H15" s="8"/>
+      <c r="I15" s="8"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="B16" s="5" t="n">
-        <v>45903</v>
+        <v>45931</v>
       </c>
       <c r="C16" s="5" t="n">
-        <v>45992</v>
+        <v>46072</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>71</v>
+        <v>18</v>
       </c>
       <c r="E16" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
+      <c r="I16" s="8"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>72</v>
+        <v>27</v>
       </c>
       <c r="B17" s="5" t="n">
-        <v>45931</v>
+        <v>46061</v>
       </c>
       <c r="C17" s="5" t="n">
-        <v>45964</v>
+        <v>46072</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>73</v>
+        <v>28</v>
       </c>
       <c r="E17" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2132,16 +2310,16 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="B18" s="5" t="n">
-        <v>45839</v>
+        <v>45993</v>
       </c>
       <c r="C18" s="5" t="n">
-        <v>45930</v>
+        <v>46060</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="E18" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2150,16 +2328,16 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>43</v>
+        <v>21</v>
       </c>
       <c r="B19" s="5" t="n">
-        <v>45839</v>
+        <v>45931</v>
       </c>
       <c r="C19" s="5" t="n">
-        <v>45930</v>
+        <v>46060</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="E19" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2168,16 +2346,16 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B20" s="5" t="n">
-        <v>45839</v>
+        <v>45903</v>
       </c>
       <c r="C20" s="5" t="n">
-        <v>45930</v>
+        <v>45992</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E20" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2186,16 +2364,16 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="B21" s="5" t="n">
-        <v>45839</v>
+        <v>45903</v>
       </c>
       <c r="C21" s="5" t="n">
-        <v>45930</v>
+        <v>45992</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="E21" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2204,16 +2382,16 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>42</v>
+        <v>77</v>
       </c>
       <c r="B22" s="5" t="n">
-        <v>45870</v>
+        <v>45931</v>
       </c>
       <c r="C22" s="5" t="n">
-        <v>45902</v>
+        <v>45964</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="E22" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2222,16 +2400,16 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>72</v>
+        <v>33</v>
       </c>
       <c r="B23" s="5" t="n">
-        <v>45870</v>
+        <v>45839</v>
       </c>
       <c r="C23" s="5" t="n">
-        <v>45902</v>
+        <v>45930</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>73</v>
+        <v>34</v>
       </c>
       <c r="E23" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2240,16 +2418,16 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B24" s="5" t="n">
-        <v>45748</v>
+        <v>45839</v>
       </c>
       <c r="C24" s="5" t="n">
-        <v>45869</v>
+        <v>45930</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E24" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2258,16 +2436,16 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>5</v>
+        <v>50</v>
       </c>
       <c r="B25" s="5" t="n">
-        <v>45653</v>
+        <v>45839</v>
       </c>
       <c r="C25" s="5" t="n">
-        <v>45869</v>
+        <v>45930</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E25" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2276,16 +2454,16 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="B26" s="5" t="n">
-        <v>45778</v>
+        <v>45839</v>
       </c>
       <c r="C26" s="5" t="n">
-        <v>45838</v>
+        <v>45930</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="E26" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2294,16 +2472,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>57</v>
+        <v>29</v>
       </c>
       <c r="B27" s="5" t="n">
-        <v>45778</v>
+        <v>45870</v>
       </c>
       <c r="C27" s="5" t="n">
-        <v>45838</v>
+        <v>45902</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="E27" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2315,10 +2493,10 @@
         <v>77</v>
       </c>
       <c r="B28" s="5" t="n">
-        <v>45778</v>
+        <v>45870</v>
       </c>
       <c r="C28" s="5" t="n">
-        <v>45838</v>
+        <v>45902</v>
       </c>
       <c r="D28" s="4" t="s">
         <v>78</v>
@@ -2330,16 +2508,16 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>55</v>
+        <v>31</v>
       </c>
       <c r="B29" s="5" t="n">
-        <v>45811</v>
+        <v>45748</v>
       </c>
       <c r="C29" s="5" t="n">
-        <v>45838</v>
+        <v>45869</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>56</v>
+        <v>32</v>
       </c>
       <c r="E29" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2348,16 +2526,16 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>79</v>
+        <v>5</v>
       </c>
       <c r="B30" s="5" t="n">
-        <v>45748</v>
+        <v>45653</v>
       </c>
       <c r="C30" s="5" t="n">
-        <v>45810</v>
+        <v>45869</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="E30" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2366,16 +2544,16 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>58</v>
+        <v>29</v>
       </c>
       <c r="B31" s="5" t="n">
-        <v>45692</v>
+        <v>45778</v>
       </c>
       <c r="C31" s="5" t="n">
-        <v>45777</v>
+        <v>45838</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E31" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2387,13 +2565,13 @@
         <v>60</v>
       </c>
       <c r="B32" s="5" t="n">
-        <v>45748</v>
+        <v>45778</v>
       </c>
       <c r="C32" s="5" t="n">
-        <v>45777</v>
+        <v>45838</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>61</v>
+        <v>81</v>
       </c>
       <c r="E32" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2405,10 +2583,10 @@
         <v>82</v>
       </c>
       <c r="B33" s="5" t="n">
-        <v>45748</v>
+        <v>45778</v>
       </c>
       <c r="C33" s="5" t="n">
-        <v>45777</v>
+        <v>45838</v>
       </c>
       <c r="D33" s="4" t="s">
         <v>83</v>
@@ -2420,16 +2598,16 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>23</v>
+        <v>58</v>
       </c>
       <c r="B34" s="5" t="n">
-        <v>45653</v>
+        <v>45811</v>
       </c>
       <c r="C34" s="5" t="n">
-        <v>45747</v>
+        <v>45838</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="E34" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2438,16 +2616,16 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>31</v>
+        <v>84</v>
       </c>
       <c r="B35" s="5" t="n">
-        <v>45653</v>
+        <v>45748</v>
       </c>
       <c r="C35" s="5" t="n">
-        <v>45747</v>
+        <v>45810</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>69</v>
+        <v>85</v>
       </c>
       <c r="E35" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2456,16 +2634,16 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
-        <v>29</v>
+        <v>61</v>
       </c>
       <c r="B36" s="5" t="n">
-        <v>45660</v>
+        <v>45692</v>
       </c>
       <c r="C36" s="5" t="n">
-        <v>45747</v>
+        <v>45777</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E36" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2474,16 +2652,16 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
-        <v>45</v>
+        <v>63</v>
       </c>
       <c r="B37" s="5" t="n">
-        <v>45660</v>
+        <v>45748</v>
       </c>
       <c r="C37" s="5" t="n">
-        <v>45747</v>
+        <v>45777</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="E37" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2492,16 +2670,16 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
-        <v>48</v>
+        <v>87</v>
       </c>
       <c r="B38" s="5" t="n">
-        <v>45660</v>
+        <v>45748</v>
       </c>
       <c r="C38" s="5" t="n">
-        <v>45747</v>
+        <v>45777</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>68</v>
+        <v>88</v>
       </c>
       <c r="E38" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2510,16 +2688,16 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B39" s="5" t="n">
-        <v>45660</v>
+        <v>45653</v>
       </c>
       <c r="C39" s="5" t="n">
-        <v>45691</v>
+        <v>45747</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>26</v>
+        <v>70</v>
       </c>
       <c r="E39" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2528,16 +2706,16 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
-        <v>17</v>
+        <v>37</v>
       </c>
       <c r="B40" s="5" t="n">
         <v>45653</v>
       </c>
       <c r="C40" s="5" t="n">
-        <v>45659</v>
+        <v>45747</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>18</v>
+        <v>74</v>
       </c>
       <c r="E40" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2546,16 +2724,16 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="s">
-        <v>85</v>
+        <v>40</v>
       </c>
       <c r="B41" s="5" t="n">
-        <v>45653</v>
+        <v>45660</v>
       </c>
       <c r="C41" s="5" t="n">
-        <v>45659</v>
+        <v>45747</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="E41" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2564,16 +2742,16 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="s">
-        <v>87</v>
+        <v>50</v>
       </c>
       <c r="B42" s="5" t="n">
-        <v>45653</v>
+        <v>45660</v>
       </c>
       <c r="C42" s="5" t="n">
-        <v>45659</v>
+        <v>45747</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="E42" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2582,36 +2760,111 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="4" t="s">
-        <v>89</v>
+        <v>53</v>
       </c>
       <c r="B43" s="5" t="n">
+        <v>45660</v>
+      </c>
+      <c r="C43" s="5" t="n">
+        <v>45747</v>
+      </c>
+      <c r="D43" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="E43" s="6" t="n">
+        <f aca="false">1/7</f>
+        <v>0.142857142857143</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>45660</v>
+      </c>
+      <c r="C44" s="5" t="n">
+        <v>45691</v>
+      </c>
+      <c r="D44" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="E44" s="6" t="n">
+        <f aca="false">1/7</f>
+        <v>0.142857142857143</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B45" s="5" t="n">
         <v>45653</v>
       </c>
-      <c r="C43" s="5" t="n">
+      <c r="C45" s="5" t="n">
         <v>45659</v>
       </c>
-      <c r="D43" s="4" t="s">
+      <c r="D45" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="E45" s="6" t="n">
+        <f aca="false">1/7</f>
+        <v>0.142857142857143</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="E43" s="6" t="n">
-        <f aca="false">1/7</f>
-        <v>0.142857142857143</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="5"/>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="5"/>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="5"/>
+      <c r="B46" s="5" t="n">
+        <v>45653</v>
+      </c>
+      <c r="C46" s="5" t="n">
+        <v>45659</v>
+      </c>
+      <c r="D46" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="E46" s="6" t="n">
+        <f aca="false">1/7</f>
+        <v>0.142857142857143</v>
+      </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="5"/>
+      <c r="A47" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>45653</v>
+      </c>
+      <c r="C47" s="5" t="n">
+        <v>45659</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="E47" s="6" t="n">
+        <f aca="false">1/7</f>
+        <v>0.142857142857143</v>
+      </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="5"/>
+      <c r="A48" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>45653</v>
+      </c>
+      <c r="C48" s="5" t="n">
+        <v>45659</v>
+      </c>
+      <c r="D48" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="E48" s="6" t="n">
+        <f aca="false">1/7</f>
+        <v>0.142857142857143</v>
+      </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="5"/>
@@ -2649,8 +2902,23 @@
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="5"/>
     </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="5"/>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="5"/>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="5"/>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="5"/>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="5"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E43"/>
+  <autoFilter ref="A1:E48"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
new comp 13 june 2026
</commit_message>
<xml_diff>
--- a/src/AlgoComposition.xlsx
+++ b/src/AlgoComposition.xlsx
@@ -14,8 +14,8 @@
     <sheet name="2015" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">'2015'!$A$1:$E$48</definedName>
-    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'2020'!$A$1:$E$48</definedName>
+    <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">'2015'!$A$1:$E$49</definedName>
+    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'2020'!$A$1:$E$49</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="96">
   <si>
     <t xml:space="preserve">Symbol</t>
   </si>
@@ -128,6 +128,9 @@
     <t xml:space="preserve">Intuit</t>
   </si>
   <si>
+    <t xml:space="preserve">Micron</t>
+  </si>
+  <si>
     <t xml:space="preserve">GRMN</t>
   </si>
   <si>
@@ -146,9 +149,6 @@
     <t xml:space="preserve">Amazon Inc.</t>
   </si>
   <si>
-    <t xml:space="preserve">Micron</t>
-  </si>
-  <si>
     <t xml:space="preserve">GOOG</t>
   </si>
   <si>
@@ -239,13 +239,13 @@
     <t xml:space="preserve">Dell</t>
   </si>
   <si>
+    <t xml:space="preserve">NVIDIA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Palantir Technologies</t>
+  </si>
+  <si>
     <t xml:space="preserve">Apple</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NVIDIA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Palantir Technologies</t>
   </si>
   <si>
     <t xml:space="preserve">PepsiCo</t>
@@ -442,7 +442,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -471,7 +471,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -481,6 +481,10 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1016,7 +1020,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J67"/>
+  <dimension ref="A1:J68"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14.02"/>
@@ -1043,10 +1047,10 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="B2" s="5" t="n">
-        <v>46175</v>
+        <v>46186</v>
       </c>
       <c r="C2" s="5" t="n">
         <v>55146</v>
@@ -1056,30 +1060,30 @@
         <v>0.142857142857143</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B3" s="5" t="n">
-        <v>46139</v>
+        <v>46175</v>
       </c>
       <c r="C3" s="5" t="n">
-        <v>55146</v>
+        <v>46185</v>
       </c>
       <c r="D3" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B4" s="5" t="n">
         <v>46139</v>
@@ -1092,25 +1096,25 @@
         <v>0.142857142857143</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="B5" s="5" t="n">
         <v>46139</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>46174</v>
+        <v>55146</v>
       </c>
       <c r="D5" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1133,118 +1137,117 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>45903</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>55146</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <f aca="false">1/7</f>
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E7" s="6" t="s">
         <v>33</v>
-      </c>
-      <c r="B7" s="5" t="n">
-        <v>46091</v>
-      </c>
-      <c r="C7" s="5" t="n">
-        <v>46138</v>
-      </c>
-      <c r="D7" s="6" t="n">
-        <f aca="false">1/7</f>
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>35</v>
+        <v>5</v>
       </c>
       <c r="B8" s="5" t="n">
-        <v>46091</v>
+        <v>45965</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>46138</v>
+        <v>55146</v>
       </c>
       <c r="D8" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="H8" s="7"/>
+        <v>6</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>37</v>
+        <v>9</v>
       </c>
       <c r="B9" s="5" t="n">
-        <v>46077</v>
+        <v>45748</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>46138</v>
+        <v>55146</v>
       </c>
       <c r="D9" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>38</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="H9" s="7"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B10" s="5" t="n">
-        <v>45903</v>
+        <v>46139</v>
       </c>
       <c r="C10" s="5" t="n">
-        <v>55146</v>
+        <v>46174</v>
       </c>
       <c r="D10" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>39</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="B11" s="5" t="n">
-        <v>45965</v>
+        <v>46091</v>
       </c>
       <c r="C11" s="5" t="n">
-        <v>55146</v>
+        <v>46138</v>
       </c>
       <c r="D11" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="I11" s="8"/>
+        <v>35</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>9</v>
+        <v>36</v>
       </c>
       <c r="B12" s="5" t="n">
-        <v>45748</v>
+        <v>46091</v>
       </c>
       <c r="C12" s="5" t="n">
-        <v>55146</v>
+        <v>46138</v>
       </c>
       <c r="D12" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="I12" s="8"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>23</v>
+        <v>38</v>
       </c>
       <c r="B13" s="5" t="n">
         <v>46077</v>
@@ -1257,33 +1260,34 @@
         <v>0.142857142857143</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>24</v>
-      </c>
+        <v>39</v>
+      </c>
+      <c r="I13" s="8"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="B14" s="5" t="n">
         <v>46077</v>
       </c>
       <c r="C14" s="5" t="n">
-        <v>46090</v>
+        <v>46138</v>
       </c>
       <c r="D14" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>41</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>13</v>
+        <v>40</v>
       </c>
       <c r="B15" s="5" t="n">
-        <v>45965</v>
+        <v>46077</v>
       </c>
       <c r="C15" s="5" t="n">
         <v>46090</v>
@@ -1293,32 +1297,31 @@
         <v>0.142857142857143</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="J15" s="8"/>
+        <v>41</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B16" s="5" t="n">
-        <v>45931</v>
+        <v>45965</v>
       </c>
       <c r="C16" s="5" t="n">
-        <v>46076</v>
+        <v>46090</v>
       </c>
       <c r="D16" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="J16" s="8"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B17" s="5" t="n">
         <v>45931</v>
@@ -1331,16 +1334,16 @@
         <v>0.142857142857143</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="J17" s="8"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="B18" s="5" t="n">
-        <v>46061</v>
+        <v>45931</v>
       </c>
       <c r="C18" s="5" t="n">
         <v>46076</v>
@@ -1350,84 +1353,85 @@
         <v>0.142857142857143</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>28</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="J18" s="8"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
       <c r="B19" s="5" t="n">
-        <v>46048</v>
+        <v>46061</v>
       </c>
       <c r="C19" s="5" t="n">
-        <v>46060</v>
+        <v>46076</v>
       </c>
       <c r="D19" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>43</v>
+        <v>28</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>21</v>
+        <v>42</v>
       </c>
       <c r="B20" s="5" t="n">
-        <v>45993</v>
+        <v>46048</v>
       </c>
       <c r="C20" s="5" t="n">
-        <v>46047</v>
+        <v>46060</v>
       </c>
       <c r="D20" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>22</v>
+        <v>43</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>44</v>
+        <v>21</v>
       </c>
       <c r="B21" s="5" t="n">
-        <v>45903</v>
+        <v>45993</v>
       </c>
       <c r="C21" s="5" t="n">
-        <v>45992</v>
+        <v>46047</v>
       </c>
       <c r="D21" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>45</v>
+        <v>22</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>19</v>
+        <v>44</v>
       </c>
       <c r="B22" s="5" t="n">
-        <v>45931</v>
+        <v>45903</v>
       </c>
       <c r="C22" s="5" t="n">
-        <v>45964</v>
+        <v>45992</v>
       </c>
       <c r="D22" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>19</v>
+        <v>45</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>46</v>
+        <v>19</v>
       </c>
       <c r="B23" s="5" t="n">
         <v>45931</v>
@@ -1440,33 +1444,33 @@
         <v>0.142857142857143</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>47</v>
+        <v>19</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>29</v>
+        <v>46</v>
       </c>
       <c r="B24" s="5" t="n">
-        <v>45778</v>
+        <v>45931</v>
       </c>
       <c r="C24" s="5" t="n">
-        <v>45930</v>
+        <v>45964</v>
       </c>
       <c r="D24" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>29</v>
+        <v>47</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B25" s="5" t="n">
-        <v>45839</v>
+        <v>45778</v>
       </c>
       <c r="C25" s="5" t="n">
         <v>45930</v>
@@ -1476,12 +1480,12 @@
         <v>0.142857142857143</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="B26" s="5" t="n">
         <v>45839</v>
@@ -1494,12 +1498,12 @@
         <v>0.142857142857143</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>49</v>
+        <v>35</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B27" s="5" t="n">
         <v>45839</v>
@@ -1512,30 +1516,30 @@
         <v>0.142857142857143</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B28" s="5" t="n">
-        <v>45870</v>
+        <v>45839</v>
       </c>
       <c r="C28" s="5" t="n">
-        <v>45902</v>
+        <v>45930</v>
       </c>
       <c r="D28" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B29" s="5" t="n">
         <v>45870</v>
@@ -1548,33 +1552,33 @@
         <v>0.142857142857143</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>31</v>
+        <v>53</v>
       </c>
       <c r="B30" s="5" t="n">
-        <v>45692</v>
+        <v>45870</v>
       </c>
       <c r="C30" s="5" t="n">
-        <v>45869</v>
+        <v>45902</v>
       </c>
       <c r="D30" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>32</v>
+        <v>54</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="B31" s="5" t="n">
-        <v>45653</v>
+        <v>45692</v>
       </c>
       <c r="C31" s="5" t="n">
         <v>45869</v>
@@ -1584,33 +1588,33 @@
         <v>0.142857142857143</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>6</v>
+        <v>32</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>55</v>
+        <v>5</v>
       </c>
       <c r="B32" s="5" t="n">
-        <v>45748</v>
+        <v>45653</v>
       </c>
       <c r="C32" s="5" t="n">
-        <v>45838</v>
+        <v>45869</v>
       </c>
       <c r="D32" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>55</v>
+        <v>6</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B33" s="5" t="n">
-        <v>45778</v>
+        <v>45748</v>
       </c>
       <c r="C33" s="5" t="n">
         <v>45838</v>
@@ -1620,15 +1624,15 @@
         <v>0.142857142857143</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B34" s="5" t="n">
-        <v>45811</v>
+        <v>45778</v>
       </c>
       <c r="C34" s="5" t="n">
         <v>45838</v>
@@ -1638,51 +1642,51 @@
         <v>0.142857142857143</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B35" s="5" t="n">
-        <v>45778</v>
+        <v>45811</v>
       </c>
       <c r="C35" s="5" t="n">
-        <v>45810</v>
+        <v>45838</v>
       </c>
       <c r="D35" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
-        <v>13</v>
+        <v>60</v>
       </c>
       <c r="B36" s="5" t="n">
-        <v>45748</v>
+        <v>45778</v>
       </c>
       <c r="C36" s="5" t="n">
-        <v>45777</v>
+        <v>45810</v>
       </c>
       <c r="D36" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>14</v>
+        <v>60</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
-        <v>61</v>
+        <v>13</v>
       </c>
       <c r="B37" s="5" t="n">
-        <v>45692</v>
+        <v>45748</v>
       </c>
       <c r="C37" s="5" t="n">
         <v>45777</v>
@@ -1692,15 +1696,15 @@
         <v>0.142857142857143</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>62</v>
+        <v>14</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B38" s="5" t="n">
-        <v>45748</v>
+        <v>45692</v>
       </c>
       <c r="C38" s="5" t="n">
         <v>45777</v>
@@ -1710,30 +1714,30 @@
         <v>0.142857142857143</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
-        <v>23</v>
+        <v>63</v>
       </c>
       <c r="B39" s="5" t="n">
-        <v>45653</v>
+        <v>45748</v>
       </c>
       <c r="C39" s="5" t="n">
-        <v>45747</v>
+        <v>45777</v>
       </c>
       <c r="D39" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>24</v>
+        <v>64</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="B40" s="5" t="n">
         <v>45653</v>
@@ -1746,15 +1750,15 @@
         <v>0.142857142857143</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>65</v>
+        <v>24</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="B41" s="5" t="n">
-        <v>45660</v>
+        <v>45653</v>
       </c>
       <c r="C41" s="5" t="n">
         <v>45747</v>
@@ -1764,12 +1768,12 @@
         <v>0.142857142857143</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>34</v>
+        <v>65</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="s">
-        <v>50</v>
+        <v>34</v>
       </c>
       <c r="B42" s="5" t="n">
         <v>45660</v>
@@ -1782,30 +1786,30 @@
         <v>0.142857142857143</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>51</v>
+        <v>35</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="4" t="s">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="B43" s="5" t="n">
         <v>45660</v>
       </c>
       <c r="C43" s="5" t="n">
-        <v>45691</v>
+        <v>45747</v>
       </c>
       <c r="D43" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E43" s="6" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="4" t="s">
-        <v>9</v>
+        <v>40</v>
       </c>
       <c r="B44" s="5" t="n">
         <v>45660</v>
@@ -1818,30 +1822,30 @@
         <v>0.142857142857143</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>10</v>
+        <v>41</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="4" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="B45" s="5" t="n">
-        <v>45653</v>
+        <v>45660</v>
       </c>
       <c r="C45" s="5" t="n">
-        <v>45659</v>
+        <v>45691</v>
       </c>
       <c r="D45" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="4" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B46" s="5" t="n">
         <v>45653</v>
@@ -1854,12 +1858,12 @@
         <v>0.142857142857143</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="4" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B47" s="5" t="n">
         <v>45653</v>
@@ -1872,12 +1876,12 @@
         <v>0.142857142857143</v>
       </c>
       <c r="E47" s="6" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="4" t="s">
-        <v>66</v>
+        <v>19</v>
       </c>
       <c r="B48" s="5" t="n">
         <v>45653</v>
@@ -1890,12 +1894,26 @@
         <v>0.142857142857143</v>
       </c>
       <c r="E48" s="6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>45653</v>
+      </c>
+      <c r="C49" s="5" t="n">
+        <v>45659</v>
+      </c>
+      <c r="D49" s="6" t="n">
+        <f aca="false">1/7</f>
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E49" s="6" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="5"/>
-      <c r="B49" s="5"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="5"/>
@@ -1969,8 +1987,12 @@
       <c r="A67" s="5"/>
       <c r="B67" s="5"/>
     </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="5"/>
+      <c r="B68" s="5"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E48"/>
+  <autoFilter ref="A1:E49"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -1987,7 +2009,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I65"/>
+  <dimension ref="A1:I66"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15.02"/>
@@ -2033,16 +2055,16 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="B3" s="5" t="n">
-        <v>46140</v>
+        <v>46186</v>
       </c>
       <c r="C3" s="5" t="n">
         <v>55146</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>32</v>
+      <c r="D3" s="10" t="s">
+        <v>14</v>
       </c>
       <c r="E3" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2051,7 +2073,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="B4" s="5" t="n">
         <v>46140</v>
@@ -2060,7 +2082,7 @@
         <v>55146</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E4" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2105,73 +2127,73 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>35</v>
+        <v>5</v>
       </c>
       <c r="B7" s="5" t="n">
-        <v>46091</v>
+        <v>45931</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>46140</v>
+        <v>55146</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>36</v>
+        <v>70</v>
       </c>
       <c r="E7" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
-      <c r="F7" s="6"/>
-      <c r="G7" s="7"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="B8" s="5" t="n">
-        <v>46091</v>
+        <v>45748</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>46140</v>
+        <v>55146</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>34</v>
+        <v>71</v>
       </c>
       <c r="E8" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
       <c r="F8" s="6"/>
+      <c r="G8" s="7"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B9" s="5" t="n">
-        <v>45965</v>
+        <v>46140</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>46140</v>
+        <v>46185</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>70</v>
+        <v>26</v>
       </c>
       <c r="E9" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
+      <c r="F9" s="6"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>5</v>
+        <v>36</v>
       </c>
       <c r="B10" s="5" t="n">
-        <v>45931</v>
+        <v>46091</v>
       </c>
       <c r="C10" s="5" t="n">
-        <v>55146</v>
+        <v>46140</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>71</v>
+        <v>37</v>
       </c>
       <c r="E10" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2180,16 +2202,16 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="B11" s="5" t="n">
-        <v>45748</v>
+        <v>46091</v>
       </c>
       <c r="C11" s="5" t="n">
-        <v>55146</v>
+        <v>46140</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>72</v>
+        <v>35</v>
       </c>
       <c r="E11" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2198,16 +2220,16 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>53</v>
+        <v>23</v>
       </c>
       <c r="B12" s="5" t="n">
-        <v>46061</v>
+        <v>45965</v>
       </c>
       <c r="C12" s="5" t="n">
         <v>46140</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E12" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2215,111 +2237,111 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5" t="s">
-        <v>37</v>
+      <c r="A13" s="4" t="s">
+        <v>53</v>
       </c>
       <c r="B13" s="5" t="n">
-        <v>46073</v>
+        <v>46061</v>
       </c>
       <c r="C13" s="5" t="n">
         <v>46140</v>
       </c>
       <c r="D13" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <f aca="false">1/7</f>
+        <v>0.142857142857143</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>46073</v>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="D14" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="E13" s="6" t="n">
-        <f aca="false">1/7</f>
-        <v>0.142857142857143</v>
-      </c>
-      <c r="H13" s="8"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
+      <c r="E14" s="6" t="n">
+        <f aca="false">1/7</f>
+        <v>0.142857142857143</v>
+      </c>
+      <c r="H14" s="8"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="5" t="n">
+      <c r="B15" s="5" t="n">
         <v>45993</v>
-      </c>
-      <c r="C14" s="5" t="n">
-        <v>46091</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E14" s="6" t="n">
-        <f aca="false">1/7</f>
-        <v>0.142857142857143</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="B15" s="5" t="n">
-        <v>46073</v>
       </c>
       <c r="C15" s="5" t="n">
         <v>46091</v>
       </c>
       <c r="D15" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15" s="6" t="n">
+        <f aca="false">1/7</f>
+        <v>0.142857142857143</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>46073</v>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>46091</v>
+      </c>
+      <c r="D16" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="E15" s="6" t="n">
-        <f aca="false">1/7</f>
-        <v>0.142857142857143</v>
-      </c>
-      <c r="H15" s="8"/>
-      <c r="I15" s="8"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B16" s="5" t="n">
-        <v>45931</v>
-      </c>
-      <c r="C16" s="5" t="n">
-        <v>46072</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>18</v>
-      </c>
       <c r="E16" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
+      <c r="H16" s="8"/>
       <c r="I16" s="8"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="B17" s="5" t="n">
-        <v>46061</v>
+        <v>45931</v>
       </c>
       <c r="C17" s="5" t="n">
         <v>46072</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="E17" s="6" t="n">
         <f aca="false">1/7</f>
         <v>0.142857142857143</v>
       </c>
+      <c r="I17" s="8"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="B18" s="5" t="n">
-        <v>45993</v>
+        <v>46061</v>
       </c>
       <c r="C18" s="5" t="n">
-        <v>46060</v>
+        <v>46072</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="E18" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2328,16 +2350,16 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="B19" s="5" t="n">
-        <v>45931</v>
+        <v>45993</v>
       </c>
       <c r="C19" s="5" t="n">
         <v>46060</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="E19" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2346,16 +2368,16 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>46</v>
+        <v>21</v>
       </c>
       <c r="B20" s="5" t="n">
-        <v>45903</v>
+        <v>45931</v>
       </c>
       <c r="C20" s="5" t="n">
-        <v>45992</v>
+        <v>46060</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>75</v>
+        <v>22</v>
       </c>
       <c r="E20" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2364,7 +2386,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B21" s="5" t="n">
         <v>45903</v>
@@ -2373,7 +2395,7 @@
         <v>45992</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E21" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2382,16 +2404,16 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>77</v>
+        <v>44</v>
       </c>
       <c r="B22" s="5" t="n">
-        <v>45931</v>
+        <v>45903</v>
       </c>
       <c r="C22" s="5" t="n">
-        <v>45964</v>
+        <v>45992</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E22" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2400,16 +2422,16 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>33</v>
+        <v>77</v>
       </c>
       <c r="B23" s="5" t="n">
-        <v>45839</v>
+        <v>45931</v>
       </c>
       <c r="C23" s="5" t="n">
-        <v>45930</v>
+        <v>45964</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>34</v>
+        <v>78</v>
       </c>
       <c r="E23" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2418,7 +2440,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="B24" s="5" t="n">
         <v>45839</v>
@@ -2427,7 +2449,7 @@
         <v>45930</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="E24" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2436,7 +2458,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B25" s="5" t="n">
         <v>45839</v>
@@ -2445,7 +2467,7 @@
         <v>45930</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>79</v>
+        <v>49</v>
       </c>
       <c r="E25" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2454,7 +2476,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B26" s="5" t="n">
         <v>45839</v>
@@ -2463,7 +2485,7 @@
         <v>45930</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="E26" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2472,16 +2494,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="B27" s="5" t="n">
-        <v>45870</v>
+        <v>45839</v>
       </c>
       <c r="C27" s="5" t="n">
-        <v>45902</v>
+        <v>45930</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="E27" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2490,7 +2512,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>77</v>
+        <v>29</v>
       </c>
       <c r="B28" s="5" t="n">
         <v>45870</v>
@@ -2499,7 +2521,7 @@
         <v>45902</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E28" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2508,16 +2530,16 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>31</v>
+        <v>77</v>
       </c>
       <c r="B29" s="5" t="n">
-        <v>45748</v>
+        <v>45870</v>
       </c>
       <c r="C29" s="5" t="n">
-        <v>45869</v>
+        <v>45902</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>32</v>
+        <v>78</v>
       </c>
       <c r="E29" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2526,16 +2548,16 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="B30" s="5" t="n">
-        <v>45653</v>
+        <v>45748</v>
       </c>
       <c r="C30" s="5" t="n">
         <v>45869</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>71</v>
+        <v>32</v>
       </c>
       <c r="E30" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2544,16 +2566,16 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="B31" s="5" t="n">
-        <v>45778</v>
+        <v>45653</v>
       </c>
       <c r="C31" s="5" t="n">
-        <v>45838</v>
+        <v>45869</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="E31" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2562,7 +2584,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>60</v>
+        <v>29</v>
       </c>
       <c r="B32" s="5" t="n">
         <v>45778</v>
@@ -2571,7 +2593,7 @@
         <v>45838</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E32" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2580,7 +2602,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>82</v>
+        <v>60</v>
       </c>
       <c r="B33" s="5" t="n">
         <v>45778</v>
@@ -2589,7 +2611,7 @@
         <v>45838</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="E33" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2598,16 +2620,16 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>58</v>
+        <v>82</v>
       </c>
       <c r="B34" s="5" t="n">
-        <v>45811</v>
+        <v>45778</v>
       </c>
       <c r="C34" s="5" t="n">
         <v>45838</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>59</v>
+        <v>83</v>
       </c>
       <c r="E34" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2616,16 +2638,16 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>84</v>
+        <v>58</v>
       </c>
       <c r="B35" s="5" t="n">
-        <v>45748</v>
+        <v>45811</v>
       </c>
       <c r="C35" s="5" t="n">
-        <v>45810</v>
+        <v>45838</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>85</v>
+        <v>59</v>
       </c>
       <c r="E35" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2634,16 +2656,16 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
-        <v>61</v>
+        <v>84</v>
       </c>
       <c r="B36" s="5" t="n">
-        <v>45692</v>
+        <v>45748</v>
       </c>
       <c r="C36" s="5" t="n">
-        <v>45777</v>
+        <v>45810</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E36" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2652,16 +2674,16 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B37" s="5" t="n">
-        <v>45748</v>
+        <v>45692</v>
       </c>
       <c r="C37" s="5" t="n">
         <v>45777</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>64</v>
+        <v>86</v>
       </c>
       <c r="E37" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2670,7 +2692,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
-        <v>87</v>
+        <v>63</v>
       </c>
       <c r="B38" s="5" t="n">
         <v>45748</v>
@@ -2679,7 +2701,7 @@
         <v>45777</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>88</v>
+        <v>64</v>
       </c>
       <c r="E38" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2688,16 +2710,16 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
-        <v>23</v>
+        <v>87</v>
       </c>
       <c r="B39" s="5" t="n">
-        <v>45653</v>
+        <v>45748</v>
       </c>
       <c r="C39" s="5" t="n">
-        <v>45747</v>
+        <v>45777</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="E39" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2706,7 +2728,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="B40" s="5" t="n">
         <v>45653</v>
@@ -2715,7 +2737,7 @@
         <v>45747</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="E40" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2724,16 +2746,16 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B41" s="5" t="n">
-        <v>45660</v>
+        <v>45653</v>
       </c>
       <c r="C41" s="5" t="n">
         <v>45747</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>89</v>
+        <v>74</v>
       </c>
       <c r="E41" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2742,7 +2764,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="B42" s="5" t="n">
         <v>45660</v>
@@ -2751,7 +2773,7 @@
         <v>45747</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="E42" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2760,7 +2782,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="4" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B43" s="5" t="n">
         <v>45660</v>
@@ -2769,7 +2791,7 @@
         <v>45747</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="E43" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2778,16 +2800,16 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="4" t="s">
-        <v>33</v>
+        <v>53</v>
       </c>
       <c r="B44" s="5" t="n">
         <v>45660</v>
       </c>
       <c r="C44" s="5" t="n">
-        <v>45691</v>
+        <v>45747</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>34</v>
+        <v>73</v>
       </c>
       <c r="E44" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2796,16 +2818,16 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="4" t="s">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="B45" s="5" t="n">
-        <v>45653</v>
+        <v>45660</v>
       </c>
       <c r="C45" s="5" t="n">
-        <v>45659</v>
+        <v>45691</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="E45" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2814,7 +2836,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="4" t="s">
-        <v>90</v>
+        <v>17</v>
       </c>
       <c r="B46" s="5" t="n">
         <v>45653</v>
@@ -2823,7 +2845,7 @@
         <v>45659</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>91</v>
+        <v>18</v>
       </c>
       <c r="E46" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2832,7 +2854,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="4" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B47" s="5" t="n">
         <v>45653</v>
@@ -2841,7 +2863,7 @@
         <v>45659</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="E47" s="6" t="n">
         <f aca="false">1/7</f>
@@ -2850,7 +2872,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="4" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B48" s="5" t="n">
         <v>45653</v>
@@ -2859,15 +2881,30 @@
         <v>45659</v>
       </c>
       <c r="D48" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="E48" s="6" t="n">
+        <f aca="false">1/7</f>
+        <v>0.142857142857143</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>45653</v>
+      </c>
+      <c r="C49" s="5" t="n">
+        <v>45659</v>
+      </c>
+      <c r="D49" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="E48" s="6" t="n">
-        <f aca="false">1/7</f>
-        <v>0.142857142857143</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="5"/>
+      <c r="E49" s="6" t="n">
+        <f aca="false">1/7</f>
+        <v>0.142857142857143</v>
+      </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="5"/>
@@ -2917,8 +2954,11 @@
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="5"/>
     </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="5"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E48"/>
+  <autoFilter ref="A1:E49"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>